<commit_message>
updated alumini photo data and buttons css
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="12150" firstSheet="10" activeTab="27"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="12150" firstSheet="21" activeTab="26"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="206">
   <si>
     <t>Year</t>
   </si>
@@ -611,7 +611,64 @@
     <t>https://media.licdn.com/dms/image/v2/C5103AQEdsBhjnc233g/profile-displayphoto-shrink_200_200/profile-displayphoto-shrink_200_200/0/1560254960329?e=2147483647&amp;v=beta&amp;t=NH0m6tvpm5uWPHOUe91O7fF8Cjl4-S4VuzNHp8vL8VQ</t>
   </si>
   <si>
-    <t>S2025/GummadiChiranjeevi</t>
+    <t xml:space="preserve">Urban Planning </t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2025/GummadiChiranjeevi</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2022/J.Jithender</t>
+  </si>
+  <si>
+    <t>Safety Analysis of Horizontal Curved</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2025/719017</t>
+  </si>
+  <si>
+    <t>K.V.R. Ravi Shankar</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2025/22CER1Q01</t>
+  </si>
+  <si>
+    <t>S.Shankar</t>
+  </si>
+  <si>
+    <t>Safety Analysis of Roundabout Intersection</t>
+  </si>
+  <si>
+    <t>Arpan Mehar</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2024/719030</t>
+  </si>
+  <si>
+    <t>Traffic Engineering</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2024/Pallela Sruthi</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2024/718106</t>
+  </si>
+  <si>
+    <t>Transportation Engineering (Rail transport Acoustics)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venkaiah Chowdary </t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2024/Khalil Ahmad Kakar</t>
+  </si>
+  <si>
+    <t>C.S.R.K Prasad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pavement Materials </t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2024/721005</t>
   </si>
 </sst>
 </file>
@@ -2104,8 +2161,17 @@
       <c r="B2" s="6" t="s">
         <v>147</v>
       </c>
+      <c r="C2" s="6" t="s">
+        <v>186</v>
+      </c>
       <c r="D2" s="3" t="s">
         <v>140</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2316,8 +2382,17 @@
       <c r="B2" t="s">
         <v>127</v>
       </c>
+      <c r="C2" t="s">
+        <v>197</v>
+      </c>
       <c r="D2" t="s">
         <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2330,6 +2405,12 @@
       <c r="D3" t="s">
         <v>121</v>
       </c>
+      <c r="E3" t="s">
+        <v>195</v>
+      </c>
+      <c r="F3" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -2338,8 +2419,17 @@
       <c r="B4" t="s">
         <v>129</v>
       </c>
+      <c r="C4" t="s">
+        <v>200</v>
+      </c>
       <c r="D4" t="s">
         <v>122</v>
+      </c>
+      <c r="E4" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2352,6 +2442,12 @@
       <c r="D5" t="s">
         <v>123</v>
       </c>
+      <c r="E5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F5" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -2363,6 +2459,9 @@
       <c r="D6" t="s">
         <v>124</v>
       </c>
+      <c r="E6" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -2374,6 +2473,9 @@
       <c r="D7" t="s">
         <v>125</v>
       </c>
+      <c r="E7" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -2382,8 +2484,17 @@
       <c r="B8" t="s">
         <v>133</v>
       </c>
+      <c r="C8" t="s">
+        <v>204</v>
+      </c>
       <c r="D8" t="s">
         <v>126</v>
+      </c>
+      <c r="E8" t="s">
+        <v>193</v>
+      </c>
+      <c r="F8" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2395,6 +2506,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="75" customWidth="1"/>
+    <col min="5" max="5" width="66.140625" customWidth="1"/>
+    <col min="6" max="6" width="32.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -2426,8 +2542,11 @@
       <c r="D2" t="s">
         <v>137</v>
       </c>
+      <c r="E2" t="s">
+        <v>193</v>
+      </c>
       <c r="F2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2437,8 +2556,17 @@
       <c r="B3" t="s">
         <v>135</v>
       </c>
+      <c r="C3" t="s">
+        <v>189</v>
+      </c>
       <c r="D3" t="s">
         <v>138</v>
+      </c>
+      <c r="E3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F3" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2448,8 +2576,17 @@
       <c r="B4" t="s">
         <v>136</v>
       </c>
+      <c r="C4" t="s">
+        <v>194</v>
+      </c>
       <c r="D4" t="s">
         <v>139</v>
+      </c>
+      <c r="E4" t="s">
+        <v>191</v>
+      </c>
+      <c r="F4" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
phd images data update
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E2E16E-6F76-4900-BAD9-0D39D0F63A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF84533A-01C0-4395-A9AC-4DFBC5116715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -676,9 +676,6 @@
     <t>Phd_Alumini/S2023/G.Shravan Kumar</t>
   </si>
   <si>
-    <t>Phd_Alumini/S2021/J.Jaya Shankar</t>
-  </si>
-  <si>
     <t>Phd_Alumini/S2021/Prashanth Shekar Lokku</t>
   </si>
   <si>
@@ -1276,6 +1273,9 @@
   </si>
   <si>
     <t xml:space="preserve">Phd_Alumini/S2020/Kaminenei Aditya </t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2021/J.Jaya Krishna</t>
   </si>
 </sst>
 </file>
@@ -1739,10 +1739,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1751,7 +1751,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -1768,7 +1768,7 @@
         <v>106</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>8</v>
@@ -1799,10 +1799,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1811,7 +1811,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -1825,10 +1825,10 @@
         <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>268</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>269</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -1863,10 +1863,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1875,7 +1875,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
@@ -1907,10 +1907,10 @@
         <v>33</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>266</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>267</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>11</v>
@@ -1944,10 +1944,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1956,7 +1956,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -1973,7 +1973,7 @@
         <v>168</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -1993,7 +1993,7 @@
         <v>169</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>39</v>
@@ -2013,7 +2013,7 @@
         <v>170</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>36</v>
@@ -2047,10 +2047,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2059,7 +2059,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2076,7 +2076,7 @@
         <v>167</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
@@ -2103,10 +2103,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2115,7 +2115,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2132,7 +2132,7 @@
         <v>166</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
@@ -2162,10 +2162,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2174,7 +2174,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2191,14 +2191,14 @@
         <v>164</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2215,7 +2215,7 @@
         <v>165</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>39</v>
@@ -2247,10 +2247,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2259,7 +2259,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="315" x14ac:dyDescent="0.25">
@@ -2280,7 +2280,7 @@
         <v>36</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2297,7 +2297,7 @@
         <v>161</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>36</v>
@@ -2328,10 +2328,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2340,7 +2340,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2357,7 +2357,7 @@
         <v>163</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2375,10 +2375,10 @@
         <v>57</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>239</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>36</v>
@@ -2412,10 +2412,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2424,7 +2424,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2441,7 +2441,7 @@
         <v>160</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2478,10 +2478,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2490,7 +2490,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2507,7 +2507,7 @@
         <v>159</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2538,10 +2538,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2550,7 +2550,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2567,16 +2567,16 @@
         <v>107</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>229</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -2604,10 +2604,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2616,7 +2616,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2633,7 +2633,7 @@
         <v>158</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>64</v>
@@ -2642,7 +2642,7 @@
         <v>65</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -2671,10 +2671,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2683,7 +2683,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2700,13 +2700,13 @@
         <v>157</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>68</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -2735,10 +2735,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2747,7 +2747,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2764,13 +2764,13 @@
         <v>151</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>71</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2787,13 +2787,13 @@
         <v>152</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2810,13 +2810,13 @@
         <v>153</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2833,7 +2833,7 @@
         <v>154</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>64</v>
@@ -2854,13 +2854,13 @@
         <v>155</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>68</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2877,7 +2877,7 @@
         <v>156</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>82</v>
@@ -2911,10 +2911,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="14" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>3</v>
@@ -2923,7 +2923,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
@@ -2942,7 +2942,7 @@
         <v>148</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>68</v>
@@ -2966,13 +2966,13 @@
         <v>149</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F3" s="12" t="s">
         <v>87</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H3" s="15"/>
       <c r="I3" s="7"/>
@@ -2992,13 +2992,13 @@
         <v>150</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>87</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H4" s="15"/>
       <c r="I4" s="7"/>
@@ -3029,10 +3029,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>3</v>
@@ -3041,7 +3041,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3058,13 +3058,13 @@
         <v>145</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>207</v>
+        <v>296</v>
       </c>
       <c r="H2" s="7"/>
     </row>
@@ -3082,13 +3082,13 @@
         <v>146</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H3" s="7"/>
     </row>
@@ -3106,13 +3106,13 @@
         <v>147</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>87</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H4" s="7"/>
     </row>
@@ -3143,10 +3143,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3155,7 +3155,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
@@ -3172,7 +3172,7 @@
         <v>137</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>71</v>
@@ -3189,13 +3189,13 @@
         <v>96</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>138</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>68</v>
@@ -3218,7 +3218,7 @@
         <v>139</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>71</v>
@@ -3239,7 +3239,7 @@
         <v>140</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>64</v>
@@ -3262,7 +3262,7 @@
         <v>141</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>64</v>
@@ -3285,7 +3285,7 @@
         <v>142</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>82</v>
@@ -3308,7 +3308,7 @@
         <v>143</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>87</v>
@@ -3344,10 +3344,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3356,7 +3356,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3370,7 +3370,7 @@
         <v>114</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F2" t="s">
         <v>194</v>
@@ -3387,10 +3387,10 @@
         <v>115</v>
       </c>
       <c r="D3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F3" t="s">
         <v>186</v>
@@ -3410,7 +3410,7 @@
         <v>116</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F4" t="s">
         <v>199</v>
@@ -3443,10 +3443,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3455,7 +3455,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -3489,7 +3489,7 @@
         <v>118</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F3" t="s">
         <v>188</v>
@@ -3512,7 +3512,7 @@
         <v>119</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F4" t="s">
         <v>194</v>
@@ -3532,7 +3532,7 @@
         <v>120</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F5" t="s">
         <v>196</v>
@@ -3552,7 +3552,7 @@
         <v>121</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F6" t="s">
         <v>188</v>
@@ -3586,7 +3586,7 @@
         <v>123</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F8" t="s">
         <v>186</v>
@@ -3616,10 +3616,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3628,7 +3628,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -3663,10 +3663,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3675,7 +3675,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -3709,7 +3709,7 @@
         <v>135</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F3" t="s">
         <v>184</v>
@@ -3732,7 +3732,7 @@
         <v>136</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F4" t="s">
         <v>184</v>
@@ -3746,22 +3746,22 @@
         <v>2025</v>
       </c>
       <c r="B5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C5" t="s">
         <v>224</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>224</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>274</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>225</v>
-      </c>
-      <c r="D5" t="s">
-        <v>225</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>292</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>275</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3769,16 +3769,16 @@
         <v>2025</v>
       </c>
       <c r="B6" t="s">
+        <v>287</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>289</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="F6" s="17" t="s">
         <v>290</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>289</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -3808,10 +3808,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3820,7 +3820,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3837,7 +3837,7 @@
         <v>108</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -3868,10 +3868,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3880,7 +3880,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3897,7 +3897,7 @@
         <v>109</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -3924,10 +3924,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3936,7 +3936,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3953,7 +3953,7 @@
         <v>110</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -3983,10 +3983,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3995,7 +3995,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -4012,7 +4012,7 @@
         <v>177</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4039,10 +4039,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4051,7 +4051,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -4068,7 +4068,7 @@
         <v>176</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4102,10 +4102,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4114,7 +4114,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="90" x14ac:dyDescent="0.25">
@@ -4140,19 +4140,19 @@
         <v>1989</v>
       </c>
       <c r="B3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D3" t="s">
         <v>175</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="L3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -4182,10 +4182,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4194,7 +4194,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -4211,7 +4211,7 @@
         <v>172</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
phd current photos update
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF84533A-01C0-4395-A9AC-4DFBC5116715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="8550" firstSheet="22" activeTab="27"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -40,8 +39,9 @@
     <sheet name="2022" sheetId="25" r:id="rId25"/>
     <sheet name="2023" sheetId="26" r:id="rId26"/>
     <sheet name="2024" sheetId="27" r:id="rId27"/>
-    <sheet name="2026" sheetId="29" r:id="rId28"/>
-    <sheet name="2025" sheetId="28" r:id="rId29"/>
+    <sheet name="2025" sheetId="28" r:id="rId28"/>
+    <sheet name="2026" sheetId="29" r:id="rId29"/>
+    <sheet name="Sheet1" sheetId="30" r:id="rId30"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="300">
   <si>
     <t>Year</t>
   </si>
@@ -440,9 +440,6 @@
   </si>
   <si>
     <t>Rama Kanth Angatha</t>
-  </si>
-  <si>
-    <t>Ramesh K</t>
   </si>
   <si>
     <t>G. Ramulu</t>
@@ -1277,11 +1274,32 @@
   <si>
     <t>Phd_Alumini/S2021/J.Jaya Krishna</t>
   </si>
+  <si>
+    <t>The primary aim of transportation is to facilitate movement of people and goods in a safe and efficient manner. To meet the objectives of transportation, there are many challenges from an engineering perspective. Among them, geometric design is the foremost requisite in planning and functional design of a roadway system. Generally, design speed is a speed used to determine the dimensions of highway geometric design elements. Many investigators have recognized that the design speed concepts, as applied to the present conditions of traffic, may not assure consistency in highway geometric design and may lead to incorrect driver expectations between successive elements of the roadway. In order to improve highway safety, the geometric design consistency evaluation is one of the promising strategies for designers.
+Present study aims to assess the horizontal alignment design consistency of two-lane rural highway sections by developing the operating speed model best suits to safety criterion design. Field data collected on 41 sites in various parts of National Highways. The geometric variables like curve radius, curve length, degree of curvature, deflection angle, and preceding tangent length are collected using total station instrument. The speed data collected at various horizontal curve sections and the preceding tangents of the curve sections are analysed to assess the 85th percentile speed of vehicle types such as Car, Motorized Two-wheeler (2W), Motorized Three-wheeler (3W), Light commercial vehicle (LCV), Trucks and Buses. The different statistical distribution analysis is carried out for speed of individual vehicle type and mixed traffic speed data. It is found that vehicle type speed data was either follows normal distribution or Log-normal distribution whereas, mixed traffic speed data follows more than one type of statistical distribution. The most common fit observed on mixed traffic speed data were Beta distribution. Thereafter, the cumulative curves of best fit distribution are drawn to estimate the 85th percentile speed.
+Pearson correlation analysis was performed between the 85th percentile speed of vehicles and geometric variables to find the strong correlated geometric variables with speed. All subset regression analysis was performed with field data and operating speed equations are established. The evaluation of geometric design consistency is performed with radius and classified curved sections to define new threshold limits suitable for all vehicle types under mixed traffic conditions. K-mean clustering analysis was performed to define threshold criteria for passenger car and heavy vehicle types. The threshold criteria used for evaluating safety level based on overall score rating of each curved section for study. The result finds the criteria proposed in present study for assessment of highway design consistency yields appropriate results with heavy vehicle class under nonuniformed traffic conditions. This study revealed that the operating speed of passenger cars at horizontal curve sections have high geometric sensitivity with radius less than 350 m, whereas the operating speed of heavy commercial vehicles showed high geometric sensitivity with radius less than 450 m.
+The difference in operating speed on curve and approach tangent sections was estimated to find the differential speeds of each vehicle type. Further, the 85th percentile speed differential (ΔV₅) estimated at a location is compared with a differential of 85th percentile operating speed (ΔV₈₅) measured at same location. Sensitivity analysis has been performed to verify the significant parameters on ΔV₅ of various vehicle types. The study develops all subset regression models to forecast operating speed reduction on horizontal curve locations by examining the relation between ΔV₅ and ΔV₈₅. The findings showed that the ΔV₈₅ undervalues ΔV₅ by 5.0 kmph, 4.0 kmph, 3.0 kmph, 6.5 kmph and 9.0 kmph for Car, 2W, 3W, LCV, and HCV, respectively. The operating speed differential model for Car is used for developing the nomograms for assessing the road geometric safety on two-lane rural highways.
+The first-order reliability method and system reliability analysis are performed by considering stopping sight distance and superelevation for estimating reliability index values and probability of non-compliance. The analysis showed a high probability of non-compliance with superelevation than the stopping sight distance as design elements. The k-means clustering analysis performed for developing safety evaluation criterion by considering the estimated reliability indices. The study defines criteria based on stopping sight distance, superelevation, and system reliability as unsafe, tolerable, and safe. Finally, the study designed calibration charts by using varying middle ordinates at various levels of probability of non-compliance for evaluating the safety consequences of different design alternatives.</t>
+  </si>
+  <si>
+    <t>This research provides a comprehensive examination of right-turn maneuvers at uncontrolled intersections. These intersections are critical points in road networks where vehicles navigate without the aid of traffic signals or signage. The research delves into several key aspects of right-turn maneuvers, including occupancy time, critical gap behavior, departure capacity, the dynamics of acceleration, and intersection delay. Data for this study was collected at ten intersections, employing videography to gather traffic data and Differential Global Positioning System (DGPS) technology to capture individual vehicle characteristics. Occupancy time analysis was conducted for both single-stage and two-stage crossings, with a specific focus on the statistical distribution of these crossing types. Single-stage crossing occupancy times typically exhibit heavy-tailed, nearly symmetrical profiles with smaller scale parameters. In contrast, two-stage crossings show higher mean values in occupancy time, displaying right-skewed distributions with prominent peaks. In a two-stage crossing scenario, the mean critical gap was found to be 1.21 times greater than that in a single-stage crossing. Two-stage crossings caused a 10% average capacity drop compared to single-stage ones. Moreover, a 10% rise in two-stage crossings led to a 40% decrease in right-turning movement capacity. Furthermore, multiple regression models were formulated to provide insights into occupancy time, departure capacity, and longitudinal and lateral acceleration/deceleration dynamics. The study introduces a new delay model for uncontrolled intersections that combined different delay components. Notably, exit delay is minimal, while turning delay contributes significantly, encompassing 72% of minor right-turn delay. Minor right-turning delay is 1.36 times the occupancy time. A novel service level gauge for minor approaches is developed using vehicle occupancy time and average volume to estimate vehicular delay. This criterion aids in evaluating uncontrolled intersection performance, enhancing traffic management and transportation planning decisions.</t>
+  </si>
+  <si>
+    <t>Ramesh  Babu  Kota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porous asphalt pavement (PAP) is designed to possess high air void contents, enabling efficient drainage of water from the pavement surface. These surfaces, including open-graded friction courses, porous friction courses, and drainage asphalt pavements, are gaining traction among organizations and industries globally. Urbanization significantly alters urban hydrology due to increased impervious surfaces, leading to stormwater runoff that introduces pollutants into nearby water bodies. Managing stormwater runoff and improving water quality in urban areas are shared objectives, often addressed through porous asphalt mixtures (PAM).
+The primary aim of this study is to investigate the impact of gradation and air void content design criteria on the drainage capacity and clogging mechanism of porous asphalt mixtures, utilizing field-collected materials from various locations and roads. Additionally, the study evaluates the performance of PAM in terms of permanent deformation, durability assessment, and stiffness parameters, considering the effect of compaction. Increased compaction levels reduce permeability and air void content, and the study compares results at each stage, calculating the refusal density value of the mixture.
+The study achieved porosity by analyzing the volumetric characteristics of aggregate packing. Aggregate shape characteristics significantly influence asphalt mix packing. A dry aggregate packing study was conducted for multiple selected gradations. Based on air void content and bulk density values, two gradations were further examined using a combination of medium viscosity binder and modified binder, and in the Open Gr-I and Gr-II packing studies, high air void content resulted from lower acceptable content, with Open Gr-II displaying higher bulk density. Following the packing studies, the Marshall Mix design procedure was used to select the optimum binder content for the four mixtures.
+Over time, the hydrological performance of permeable pavements degrades due to surface clogging from material accumulation. Evaluating the extent of surface clogging is crucial for determining permeable pavements' effectiveness and absorbed permeability. Location, site characteristics, and rain event frequency influence clogging rates. This study employed four different mixtures, creating samples exposed to simulated stormwater events to elucidate relationships between physical components and surface clogging development. Artificial neural network (ANN) models analysed and predicted clogging progression rates, examining the impact of aggregate gradation on permeability, sample thickness, and clogging material value.
+Regarding permanent deformation characteristics, a modified binder mixture exhibited high rut depths of 2.5 to 5.2 mm at different temperatures and mixtures. The VG30 binder showed a maximum rut depth of 12.2 mm in Open Gr-I and lower values at 50°C in Open Gr-II. Durability assessments revealed that both binders performed well, meeting the Cantabro loss limit. The porous asphalt mixture's resilient modulus value exceeded 2400 MPa, with the modified binders showing the highest values.
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1717,7 +1735,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1739,10 +1757,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1751,7 +1769,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -1768,7 +1786,7 @@
         <v>106</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>8</v>
@@ -1780,7 +1798,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1799,10 +1817,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1811,7 +1829,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -1825,10 +1843,10 @@
         <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>267</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>268</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -1843,7 +1861,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1863,10 +1881,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1875,7 +1893,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
@@ -1889,7 +1907,7 @@
         <v>31</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
@@ -1907,16 +1925,16 @@
         <v>33</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>265</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>266</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -1925,7 +1943,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1944,10 +1962,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1956,7 +1974,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -1970,10 +1988,10 @@
         <v>35</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -1990,10 +2008,10 @@
         <v>38</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>39</v>
@@ -2010,10 +2028,10 @@
         <v>41</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>36</v>
@@ -2029,7 +2047,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2047,10 +2065,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2059,7 +2077,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2073,10 +2091,10 @@
         <v>43</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
@@ -2088,7 +2106,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2103,10 +2121,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2115,7 +2133,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2129,10 +2147,10 @@
         <v>45</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
@@ -2144,7 +2162,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2162,10 +2180,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2174,7 +2192,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2188,17 +2206,17 @@
         <v>47</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2212,10 +2230,10 @@
         <v>49</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>39</v>
@@ -2228,7 +2246,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2247,10 +2265,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2259,7 +2277,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="315" x14ac:dyDescent="0.25">
@@ -2273,14 +2291,14 @@
         <v>51</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2294,10 +2312,10 @@
         <v>53</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>36</v>
@@ -2310,7 +2328,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2328,10 +2346,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2340,7 +2358,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2354,10 +2372,10 @@
         <v>55</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2375,10 +2393,10 @@
         <v>57</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>238</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>36</v>
@@ -2391,7 +2409,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2412,10 +2430,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2424,7 +2442,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2438,10 +2456,10 @@
         <v>59</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2457,7 +2475,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2478,10 +2496,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2490,7 +2508,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2504,10 +2522,10 @@
         <v>61</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2520,7 +2538,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2538,10 +2556,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2550,7 +2568,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2567,16 +2585,16 @@
         <v>107</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -2585,7 +2603,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2604,10 +2622,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2616,7 +2634,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2630,10 +2648,10 @@
         <v>63</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>64</v>
@@ -2642,7 +2660,7 @@
         <v>65</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -2651,7 +2669,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2671,10 +2689,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2683,7 +2701,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2697,16 +2715,16 @@
         <v>67</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>68</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -2715,7 +2733,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2735,10 +2753,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2747,7 +2765,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2761,16 +2779,16 @@
         <v>70</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>71</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2784,16 +2802,16 @@
         <v>73</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2807,16 +2825,16 @@
         <v>75</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2830,10 +2848,10 @@
         <v>77</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>64</v>
@@ -2851,16 +2869,16 @@
         <v>79</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>68</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -2874,10 +2892,10 @@
         <v>81</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>82</v>
@@ -2890,7 +2908,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2911,10 +2929,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="14" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>3</v>
@@ -2923,7 +2941,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
@@ -2939,10 +2957,10 @@
         <v>84</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>68</v>
@@ -2963,16 +2981,16 @@
         <v>86</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F3" s="12" t="s">
         <v>87</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H3" s="15"/>
       <c r="I3" s="7"/>
@@ -2989,16 +3007,16 @@
         <v>89</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>87</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H4" s="15"/>
       <c r="I4" s="7"/>
@@ -3010,7 +3028,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3029,10 +3047,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>3</v>
@@ -3041,7 +3059,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3055,16 +3073,16 @@
         <v>91</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H2" s="7"/>
     </row>
@@ -3079,16 +3097,16 @@
         <v>93</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H3" s="7"/>
     </row>
@@ -3103,16 +3121,16 @@
         <v>95</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>87</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H4" s="7"/>
     </row>
@@ -3122,7 +3140,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3143,10 +3161,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3155,7 +3173,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
@@ -3163,22 +3181,22 @@
         <v>2022</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>71</v>
       </c>
       <c r="G2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3189,19 +3207,19 @@
         <v>96</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>68</v>
       </c>
       <c r="G3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3215,10 +3233,10 @@
         <v>98</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>71</v>
@@ -3236,16 +3254,16 @@
         <v>100</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3259,16 +3277,16 @@
         <v>102</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3282,16 +3300,16 @@
         <v>104</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>82</v>
       </c>
       <c r="G7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3299,22 +3317,22 @@
         <v>2022</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>105</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>87</v>
       </c>
       <c r="G8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -3323,7 +3341,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3344,10 +3362,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3356,7 +3374,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3370,10 +3388,10 @@
         <v>114</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3387,16 +3405,16 @@
         <v>115</v>
       </c>
       <c r="D3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3410,10 +3428,10 @@
         <v>116</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -3422,7 +3440,7 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3443,10 +3461,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3455,10 +3473,10 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -3466,16 +3484,19 @@
         <v>124</v>
       </c>
       <c r="C2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D2" t="s">
         <v>117</v>
       </c>
+      <c r="E2" s="10" t="s">
+        <v>296</v>
+      </c>
       <c r="F2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G2" t="s">
         <v>188</v>
-      </c>
-      <c r="G2" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3489,13 +3510,13 @@
         <v>118</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3506,19 +3527,19 @@
         <v>126</v>
       </c>
       <c r="C4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D4" t="s">
         <v>119</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3532,13 +3553,13 @@
         <v>120</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3552,24 +3573,27 @@
         <v>121</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F6" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2024</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>298</v>
       </c>
       <c r="D7" t="s">
         <v>122</v>
       </c>
+      <c r="E7" s="15" t="s">
+        <v>297</v>
+      </c>
       <c r="F7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3577,22 +3601,22 @@
         <v>2024</v>
       </c>
       <c r="B8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D8" t="s">
         <v>123</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3601,46 +3625,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E2" s="10"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3663,10 +3648,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3675,24 +3660,27 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>134</v>
+        <v>133</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>299</v>
       </c>
       <c r="F2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3700,22 +3688,22 @@
         <v>2025</v>
       </c>
       <c r="B3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="F3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G3" t="s">
         <v>182</v>
-      </c>
-      <c r="D3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="F3" t="s">
-        <v>184</v>
-      </c>
-      <c r="G3" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3723,22 +3711,22 @@
         <v>2025</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F4" t="s">
+        <v>183</v>
+      </c>
+      <c r="G4" t="s">
         <v>184</v>
-      </c>
-      <c r="G4" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3746,22 +3734,22 @@
         <v>2025</v>
       </c>
       <c r="B5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C5" t="s">
         <v>223</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>223</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>224</v>
-      </c>
-      <c r="D5" t="s">
-        <v>224</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>291</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>274</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3769,28 +3757,67 @@
         <v>2025</v>
       </c>
       <c r="B6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="F6" s="17" t="s">
         <v>289</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>290</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-1C00-000000000000}"/>
+    <hyperlink ref="G5" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E2" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3808,10 +3835,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3820,7 +3847,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3837,7 +3864,7 @@
         <v>108</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -3848,8 +3875,17 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3868,10 +3904,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3880,7 +3916,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3897,7 +3933,7 @@
         <v>109</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -3909,7 +3945,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3924,10 +3960,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3936,7 +3972,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3953,7 +3989,7 @@
         <v>110</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -3965,7 +4001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3983,10 +4019,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3995,7 +4031,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -4009,10 +4045,10 @@
         <v>19</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4024,7 +4060,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4039,10 +4075,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4051,7 +4087,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -4065,10 +4101,10 @@
         <v>21</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4080,7 +4116,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4102,10 +4138,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4114,7 +4150,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="90" x14ac:dyDescent="0.25">
@@ -4128,7 +4164,7 @@
         <v>23</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
@@ -4140,19 +4176,19 @@
         <v>1989</v>
       </c>
       <c r="B3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="L3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -4161,7 +4197,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4182,10 +4218,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4194,7 +4230,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -4208,10 +4244,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4228,7 +4264,7 @@
         <v>27</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">

</xml_diff>

<commit_message>
phd data update and placements graph
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\mainnn\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="8550" firstSheet="22" activeTab="27"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="8550" firstSheet="20" activeTab="22"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="304">
   <si>
     <t>Year</t>
   </si>
@@ -1294,6 +1294,18 @@
 Over time, the hydrological performance of permeable pavements degrades due to surface clogging from material accumulation. Evaluating the extent of surface clogging is crucial for determining permeable pavements' effectiveness and absorbed permeability. Location, site characteristics, and rain event frequency influence clogging rates. This study employed four different mixtures, creating samples exposed to simulated stormwater events to elucidate relationships between physical components and surface clogging development. Artificial neural network (ANN) models analysed and predicted clogging progression rates, examining the impact of aggregate gradation on permeability, sample thickness, and clogging material value.
 Regarding permanent deformation characteristics, a modified binder mixture exhibited high rut depths of 2.5 to 5.2 mm at different temperatures and mixtures. The VG30 binder showed a maximum rut depth of 12.2 mm in Open Gr-I and lower values at 50°C in Open Gr-II. Durability assessments revealed that both binders performed well, meeting the Cantabro loss limit. The porous asphalt mixture's resilient modulus value exceeded 2400 MPa, with the modified binders showing the highest values.
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phd_Alumini/S2025/S. Padma Tejaswi </t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2024/Ramesh Babu Kota</t>
+  </si>
+  <si>
+    <t>Previous Faculty/B.P.Chandrashekhar</t>
+  </si>
+  <si>
+    <t>Previous Faculty/TS Reddy</t>
   </si>
 </sst>
 </file>
@@ -1420,7 +1432,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1455,6 +1467,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1868,6 +1881,7 @@
     <col min="4" max="4" width="21.85546875" customWidth="1"/>
     <col min="5" max="5" width="44.140625" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1912,6 +1926,9 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3594,6 +3611,9 @@
       </c>
       <c r="F7" t="s">
         <v>187</v>
+      </c>
+      <c r="G7" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3767,6 +3787,9 @@
       </c>
       <c r="F6" s="17" t="s">
         <v>289</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -3938,6 +3961,9 @@
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="G2" s="3" t="s">
+        <v>302</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
phd alumini data update
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\mainnn\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Documents\PA_catts(A)\mainnn\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="8550" firstSheet="23" activeTab="28"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" firstSheet="11" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="320">
   <si>
     <t>Year</t>
   </si>
@@ -1339,12 +1339,33 @@
   <si>
     <t>Development of User centric Transit Ecosystem Index (TEI): A Framework for Integrating Optimized Level of Service and Desirability Score of Transit Accessing Infrastructure.</t>
   </si>
+  <si>
+    <t>Transportation Engineering</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2024/ANGATHA RAMA KANTH</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2023/T. Arjun Kumar</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2022/Pallavi G</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S2019/P. Sharat Chandra</t>
+  </si>
+  <si>
+    <t>Phd_Alumini/S1998/R. Murugesan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Professor (Department of Civil Engineering) at Nandha Engineering College Erode, Tamil Nadu </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="17">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1457,6 +1478,12 @@
       <color theme="10"/>
       <name val="Times New Roman "/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1479,7 +1506,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1522,6 +1549,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1804,7 +1832,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
     <col min="3" max="5" width="42.28515625" customWidth="1"/>
@@ -1813,7 +1841,7 @@
     <col min="8" max="8" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1839,7 +1867,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1980</v>
       </c>
@@ -1867,14 +1895,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="21.42578125" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="7" max="7" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1900,7 +1928,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1996</v>
       </c>
@@ -1923,7 +1951,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75">
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G3" s="2"/>
     </row>
   </sheetData>
@@ -1934,7 +1962,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="21.85546875" customWidth="1"/>
     <col min="5" max="5" width="44.140625" customWidth="1"/>
@@ -1942,7 +1970,7 @@
     <col min="7" max="7" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1968,7 +1996,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="60">
+    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1997</v>
       </c>
@@ -1989,7 +2017,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1997</v>
       </c>
@@ -2020,13 +2048,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="5" max="5" width="157.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2052,7 +2080,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1998</v>
       </c>
@@ -2071,8 +2099,14 @@
       <c r="F2" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="409.5">
+      <c r="G2" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="H2" s="24" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1998</v>
       </c>
@@ -2092,7 +2126,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>1998</v>
       </c>
@@ -2112,7 +2146,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
     </row>
@@ -2124,12 +2158,12 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2155,7 +2189,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1999</v>
       </c>
@@ -2183,9 +2217,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2211,7 +2245,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2000</v>
       </c>
@@ -2239,12 +2273,12 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2270,7 +2304,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2001</v>
       </c>
@@ -2294,7 +2328,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2001</v>
       </c>
@@ -2323,13 +2357,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="60.28515625" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2355,7 +2389,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="315">
+    <row r="2" spans="1:8" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2003</v>
       </c>
@@ -2376,7 +2410,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2003</v>
       </c>
@@ -2405,12 +2439,12 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2436,7 +2470,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2004</v>
       </c>
@@ -2457,7 +2491,7 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2004</v>
       </c>
@@ -2486,7 +2520,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="24.7109375" customWidth="1"/>
     <col min="4" max="4" width="23.42578125" customWidth="1"/>
@@ -2494,7 +2528,7 @@
     <col min="6" max="6" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2520,7 +2554,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2005</v>
       </c>
@@ -2541,7 +2575,7 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75">
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G3" s="2"/>
     </row>
   </sheetData>
@@ -2552,7 +2586,7 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.5703125" customWidth="1"/>
     <col min="3" max="3" width="27.7109375" customWidth="1"/>
@@ -2560,7 +2594,7 @@
     <col min="5" max="5" width="48.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2586,7 +2620,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2006</v>
       </c>
@@ -2615,12 +2649,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="5" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2646,7 +2680,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1982</v>
       </c>
@@ -2680,13 +2714,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="45.5703125" customWidth="1"/>
     <col min="8" max="8" width="40.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2712,7 +2746,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2012</v>
       </c>
@@ -2746,14 +2780,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="4" max="4" width="30.42578125" customWidth="1"/>
     <col min="5" max="5" width="58.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2779,7 +2813,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2018</v>
       </c>
@@ -2810,14 +2844,14 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="138.5703125" customWidth="1"/>
     <col min="6" max="6" width="16.42578125" customWidth="1"/>
     <col min="7" max="7" width="40.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2843,7 +2877,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2019</v>
       </c>
@@ -2866,7 +2900,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2019</v>
       </c>
@@ -2889,7 +2923,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2019</v>
       </c>
@@ -2912,7 +2946,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="409.5">
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>2019</v>
       </c>
@@ -2931,9 +2965,11 @@
       <c r="F5" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="409.5">
+      <c r="G5" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>2019</v>
       </c>
@@ -2956,7 +2992,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="409.5">
+    <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>2019</v>
       </c>
@@ -2987,7 +3023,7 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34.140625" customWidth="1"/>
     <col min="3" max="3" width="56.140625" customWidth="1"/>
@@ -2995,7 +3031,7 @@
     <col min="5" max="5" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -3023,7 +3059,7 @@
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
     </row>
-    <row r="2" spans="1:10" ht="409.5">
+    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="12">
         <v>2020</v>
       </c>
@@ -3049,7 +3085,7 @@
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
     </row>
-    <row r="3" spans="1:10" ht="409.5">
+    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="12">
         <v>2020</v>
       </c>
@@ -3075,7 +3111,7 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
     </row>
-    <row r="4" spans="1:10" ht="409.5">
+    <row r="4" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>2020</v>
       </c>
@@ -3109,13 +3145,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="39.7109375" customWidth="1"/>
     <col min="5" max="5" width="118.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -3141,7 +3177,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>2021</v>
       </c>
@@ -3165,7 +3201,7 @@
       </c>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2021</v>
       </c>
@@ -3189,7 +3225,7 @@
       </c>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>2021</v>
       </c>
@@ -3221,7 +3257,7 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.42578125" customWidth="1"/>
     <col min="3" max="4" width="41.5703125" customWidth="1"/>
@@ -3229,7 +3265,7 @@
     <col min="6" max="6" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3255,7 +3291,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.5">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2022</v>
       </c>
@@ -3278,7 +3314,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2022</v>
       </c>
@@ -3301,7 +3337,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2022</v>
       </c>
@@ -3320,9 +3356,11 @@
       <c r="F4" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="409.5">
+      <c r="G4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>2022</v>
       </c>
@@ -3345,7 +3383,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="409.5">
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>2022</v>
       </c>
@@ -3368,7 +3406,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="409.5">
+    <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>2022</v>
       </c>
@@ -3391,7 +3429,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="409.5">
+    <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>2022</v>
       </c>
@@ -3422,7 +3460,7 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.28515625" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
@@ -3430,7 +3468,7 @@
     <col min="6" max="6" width="70.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3456,7 +3494,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2023</v>
       </c>
@@ -3472,8 +3510,11 @@
       <c r="F2" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="409.5">
+      <c r="G2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2023</v>
       </c>
@@ -3496,7 +3537,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2023</v>
       </c>
@@ -3521,7 +3562,7 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="51.85546875" customWidth="1"/>
     <col min="4" max="4" width="45.5703125" customWidth="1"/>
@@ -3529,7 +3570,7 @@
     <col min="6" max="6" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3555,7 +3596,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -3578,7 +3619,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -3598,7 +3639,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2024</v>
       </c>
@@ -3621,7 +3662,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="409.5">
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -3641,13 +3682,16 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="409.5">
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2024</v>
       </c>
       <c r="B6" t="s">
         <v>128</v>
       </c>
+      <c r="C6" t="s">
+        <v>313</v>
+      </c>
       <c r="D6" t="s">
         <v>121</v>
       </c>
@@ -3657,8 +3701,11 @@
       <c r="F6" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75">
+      <c r="G6" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2024</v>
       </c>
@@ -3678,7 +3725,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="409.5">
+    <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -3709,7 +3756,7 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.28515625" customWidth="1"/>
     <col min="3" max="3" width="54" customWidth="1"/>
@@ -3719,7 +3766,7 @@
     <col min="8" max="8" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3745,7 +3792,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -3765,7 +3812,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -3788,7 +3835,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2025</v>
       </c>
@@ -3811,7 +3858,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="409.5">
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2025</v>
       </c>
@@ -3834,7 +3881,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="409.5">
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -3865,14 +3912,14 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.140625" customWidth="1"/>
     <col min="3" max="3" width="38.140625" customWidth="1"/>
     <col min="5" max="5" width="36.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3898,7 +3945,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -3932,12 +3979,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="48.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3963,7 +4010,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1983</v>
       </c>
@@ -3991,13 +4038,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10.140625" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4023,7 +4070,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1984</v>
       </c>
@@ -4054,9 +4101,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4082,7 +4129,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1985</v>
       </c>
@@ -4110,12 +4157,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="93.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4141,7 +4188,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1986</v>
       </c>
@@ -4169,9 +4216,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4197,7 +4244,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1988</v>
       </c>
@@ -4225,7 +4272,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.42578125" customWidth="1"/>
     <col min="3" max="3" width="23.7109375" customWidth="1"/>
@@ -4234,7 +4281,7 @@
     <col min="6" max="6" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4260,7 +4307,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="90">
+    <row r="2" spans="1:12" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1989</v>
       </c>
@@ -4278,7 +4325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="409.5">
+    <row r="3" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1989</v>
       </c>
@@ -4306,7 +4353,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="30.7109375" customWidth="1"/>
     <col min="4" max="4" width="42" customWidth="1"/>
@@ -4314,7 +4361,7 @@
     <col min="6" max="6" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4340,7 +4387,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1992</v>
       </c>
@@ -4360,7 +4407,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="60">
+    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1992</v>
       </c>

</xml_diff>

<commit_message>
mtech and phd data update
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" firstSheet="2" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" firstSheet="5" activeTab="22"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -3098,16 +3098,19 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="34.140625" customWidth="1"/>
     <col min="3" max="3" width="56.140625" customWidth="1"/>
     <col min="4" max="4" width="53.28515625" customWidth="1"/>
     <col min="5" max="5" width="46.5703125" customWidth="1"/>
+    <col min="6" max="6" width="42.85546875" customWidth="1"/>
+    <col min="7" max="7" width="48.7109375" customWidth="1"/>
+    <col min="8" max="8" width="67" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75">
+    <row r="1" spans="1:8" ht="15.75">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -3132,10 +3135,8 @@
       <c r="H1" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-    </row>
-    <row r="2" spans="1:10" ht="409.5">
+    </row>
+    <row r="2" spans="1:8" ht="409.5">
       <c r="A2" s="12">
         <v>2020</v>
       </c>
@@ -3157,11 +3158,8 @@
       <c r="G2" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-    </row>
-    <row r="3" spans="1:10" ht="409.5">
+    </row>
+    <row r="3" spans="1:8" ht="409.5">
       <c r="A3" s="12">
         <v>2020</v>
       </c>
@@ -3183,11 +3181,8 @@
       <c r="G3" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="1:10" ht="409.5">
+    </row>
+    <row r="4" spans="1:8" ht="409.5">
       <c r="A4" s="12">
         <v>2020</v>
       </c>
@@ -3209,9 +3204,6 @@
       <c r="G4" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="H4" s="15"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>